<commit_message>
chore: update planning checklist spreadsheet
</commit_message>
<xml_diff>
--- a/docs/static/examples/tf/accelerator/config/checklist.xlsx
+++ b/docs/static/examples/tf/accelerator/config/checklist.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\ALZ\Azure-Landing-Zones\docs\static\examples\tf\accelerator\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Q:\Code\azure-landing-zones\docs\static\examples\tf\accelerator\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FC32A13-BE42-45CD-BF78-974C9F6E3F31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AE11738-6F5E-492B-A1B1-CABE6362F3B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="415" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" tabRatio="415" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Accelerator - Bootstrap" sheetId="13" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="192">
   <si>
     <t>Description</t>
   </si>
@@ -599,6 +599,30 @@
   <si>
     <t>bicep
 terraform</t>
+  </si>
+  <si>
+    <t>Change Firewall SKU</t>
+  </si>
+  <si>
+    <t>Do you want to downgrade the Firewall SKU?</t>
+  </si>
+  <si>
+    <t>Create and Assign Custom Policies</t>
+  </si>
+  <si>
+    <t>Do you want to create and assign Custom Policies?</t>
+  </si>
+  <si>
+    <t>SMB Single-Region Hub and Spoke Virtual Network with Azure Firewall</t>
+  </si>
+  <si>
+    <t>SMB Single-Region Virtual WAN with Azure Firewall</t>
+  </si>
+  <si>
+    <t>A cost-optimized platform landing zone for small-medium businesses using hub and spoke Virtual Network connectivity with Azure Firewall in a single region.</t>
+  </si>
+  <si>
+    <t>A cost-optimized platform landing zone for small-medium businesses using Virtual WAN connectivity with Azure Firewall in a single region.</t>
   </si>
 </sst>
 </file>
@@ -795,6 +819,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1061,17 +1089,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D33EA6D-E1B5-4751-908D-ADA676A42D17}">
   <dimension ref="A1:G45"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" style="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="42.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="39.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.81640625" style="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="42.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="39.81640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="38" customWidth="1"/>
-    <col min="5" max="5" width="50.42578125" customWidth="1"/>
-    <col min="6" max="7" width="46.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="50.453125" customWidth="1"/>
+    <col min="6" max="7" width="46.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="77.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="77.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="21" t="s">
         <v>155</v>
       </c>
@@ -1082,7 +1110,7 @@
       <c r="F1" s="21"/>
       <c r="G1" s="21"/>
     </row>
-    <row r="3" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="14" t="s">
         <v>157</v>
       </c>
@@ -1105,7 +1133,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="13">
         <v>1</v>
       </c>
@@ -1124,7 +1152,7 @@
       <c r="F4" s="8"/>
       <c r="G4" s="4"/>
     </row>
-    <row r="5" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A5" s="13">
         <v>2</v>
       </c>
@@ -1143,7 +1171,7 @@
       <c r="F5" s="5"/>
       <c r="G5" s="4"/>
     </row>
-    <row r="6" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A6" s="13">
         <v>3</v>
       </c>
@@ -1164,7 +1192,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="15"/>
       <c r="B7" s="6"/>
       <c r="C7" s="7"/>
@@ -1173,7 +1201,7 @@
       <c r="F7" s="6"/>
       <c r="G7" s="6"/>
     </row>
-    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="13">
         <v>4</v>
       </c>
@@ -1194,7 +1222,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A9" s="13">
         <v>6</v>
       </c>
@@ -1215,7 +1243,7 @@
       </c>
       <c r="G9" s="4"/>
     </row>
-    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="13">
         <v>7</v>
       </c>
@@ -1234,7 +1262,7 @@
       <c r="F10" s="5"/>
       <c r="G10" s="4"/>
     </row>
-    <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="13">
         <v>7</v>
       </c>
@@ -1253,7 +1281,7 @@
       <c r="F11" s="5"/>
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="13">
         <v>7</v>
       </c>
@@ -1272,7 +1300,7 @@
       <c r="F12" s="5"/>
       <c r="G12" s="4"/>
     </row>
-    <row r="13" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="13">
         <v>7</v>
       </c>
@@ -1291,7 +1319,7 @@
       <c r="F13" s="18"/>
       <c r="G13" s="4"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="15"/>
       <c r="B14" s="6"/>
       <c r="C14" s="7"/>
@@ -1300,7 +1328,7 @@
       <c r="F14" s="6"/>
       <c r="G14" s="6"/>
     </row>
-    <row r="15" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="13">
         <v>8</v>
       </c>
@@ -1321,7 +1349,7 @@
       </c>
       <c r="G15" s="4"/>
     </row>
-    <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="13">
         <v>9</v>
       </c>
@@ -1342,7 +1370,7 @@
       </c>
       <c r="G16" s="4"/>
     </row>
-    <row r="17" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="13">
         <v>9</v>
       </c>
@@ -1363,7 +1391,7 @@
       </c>
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="13">
         <v>9</v>
       </c>
@@ -1384,7 +1412,7 @@
       </c>
       <c r="G18" s="4"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="15"/>
       <c r="B19" s="6"/>
       <c r="C19" s="7"/>
@@ -1393,7 +1421,7 @@
       <c r="F19" s="6"/>
       <c r="G19" s="6"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="16"/>
       <c r="B20" s="9" t="s">
         <v>85</v>
@@ -1404,7 +1432,7 @@
       <c r="F20" s="6"/>
       <c r="G20" s="6"/>
     </row>
-    <row r="21" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A21" s="13">
         <v>11</v>
       </c>
@@ -1425,7 +1453,7 @@
       </c>
       <c r="G21" s="4"/>
     </row>
-    <row r="22" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A22" s="13">
         <v>10</v>
       </c>
@@ -1446,7 +1474,7 @@
       </c>
       <c r="G22" s="4"/>
     </row>
-    <row r="23" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A23" s="13"/>
       <c r="B23" s="4" t="s">
         <v>92</v>
@@ -1465,7 +1493,7 @@
       </c>
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A24" s="13">
         <v>11</v>
       </c>
@@ -1486,7 +1514,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A25" s="13">
         <v>11</v>
       </c>
@@ -1507,7 +1535,7 @@
       </c>
       <c r="G25" s="4"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="15"/>
       <c r="B26" s="6"/>
       <c r="C26" s="7"/>
@@ -1516,7 +1544,7 @@
       <c r="F26" s="6"/>
       <c r="G26" s="6"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="16"/>
       <c r="B27" s="9" t="s">
         <v>84</v>
@@ -1527,7 +1555,7 @@
       <c r="F27" s="6"/>
       <c r="G27" s="6"/>
     </row>
-    <row r="28" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A28" s="13">
         <v>11</v>
       </c>
@@ -1544,7 +1572,7 @@
       <c r="F28" s="5"/>
       <c r="G28" s="4"/>
     </row>
-    <row r="29" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A29" s="13">
         <v>11</v>
       </c>
@@ -1561,7 +1589,7 @@
       <c r="F29" s="5"/>
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="13">
         <v>11</v>
       </c>
@@ -1578,7 +1606,7 @@
       <c r="F30" s="5"/>
       <c r="G30" s="4"/>
     </row>
-    <row r="31" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A31" s="13">
         <v>11</v>
       </c>
@@ -1599,7 +1627,7 @@
       </c>
       <c r="G31" s="4"/>
     </row>
-    <row r="32" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A32" s="13">
         <v>11</v>
       </c>
@@ -1620,7 +1648,7 @@
       </c>
       <c r="G32" s="4"/>
     </row>
-    <row r="33" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A33" s="13">
         <v>11</v>
       </c>
@@ -1637,7 +1665,7 @@
       <c r="F33" s="5"/>
       <c r="G33" s="4"/>
     </row>
-    <row r="34" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A34" s="13">
         <v>10</v>
       </c>
@@ -1656,7 +1684,7 @@
       </c>
       <c r="G34" s="4"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" s="15"/>
       <c r="B35" s="6"/>
       <c r="C35" s="7"/>
@@ -1665,7 +1693,7 @@
       <c r="F35" s="6"/>
       <c r="G35" s="6"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="16"/>
       <c r="B36" s="9" t="s">
         <v>86</v>
@@ -1676,7 +1704,7 @@
       <c r="F36" s="6"/>
       <c r="G36" s="6"/>
     </row>
-    <row r="37" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A37" s="13">
         <v>11</v>
       </c>
@@ -1693,7 +1721,7 @@
       <c r="F37" s="5"/>
       <c r="G37" s="4"/>
     </row>
-    <row r="38" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A38" s="13">
         <v>11</v>
       </c>
@@ -1710,7 +1738,7 @@
       <c r="F38" s="5"/>
       <c r="G38" s="4"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" s="13">
         <v>11</v>
       </c>
@@ -1727,7 +1755,7 @@
       <c r="F39" s="5"/>
       <c r="G39" s="4"/>
     </row>
-    <row r="40" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A40" s="13">
         <v>10</v>
       </c>
@@ -1746,7 +1774,7 @@
       </c>
       <c r="G40" s="4"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" s="15"/>
       <c r="B41" s="6"/>
       <c r="C41" s="7"/>
@@ -1755,7 +1783,7 @@
       <c r="F41" s="6"/>
       <c r="G41" s="6"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" s="16"/>
       <c r="B42" s="9" t="s">
         <v>73</v>
@@ -1766,7 +1794,7 @@
       <c r="F42" s="6"/>
       <c r="G42" s="6"/>
     </row>
-    <row r="43" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A43" s="13">
         <v>11</v>
       </c>
@@ -1787,7 +1815,7 @@
       </c>
       <c r="G43" s="4"/>
     </row>
-    <row r="44" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A44" s="13">
         <v>11</v>
       </c>
@@ -1808,7 +1836,7 @@
       </c>
       <c r="G44" s="4"/>
     </row>
-    <row r="45" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A45" s="13">
         <v>11</v>
       </c>
@@ -1841,19 +1869,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA5559C7-55D7-4845-9950-8EEEDB97C0FA}">
   <dimension ref="A1:G30"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="47.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="47.54296875" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="44" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.5703125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="17.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.54296875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="17.453125" style="3" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="2"/>
+    <col min="6" max="6" width="13.26953125" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.54296875" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.1796875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="20" t="s">
         <v>181</v>
       </c>
@@ -1864,7 +1892,7 @@
       <c r="F1" s="20"/>
       <c r="G1" s="20"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2"/>
       <c r="B2"/>
       <c r="C2"/>
@@ -1873,7 +1901,7 @@
       <c r="F2"/>
       <c r="G2"/>
     </row>
-    <row r="3" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="11" t="s">
         <v>165</v>
       </c>
@@ -1896,7 +1924,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="6"/>
       <c r="B4" s="6"/>
       <c r="C4" s="7"/>
@@ -1905,7 +1933,7 @@
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
         <v>148</v>
       </c>
@@ -1916,7 +1944,7 @@
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
     </row>
-    <row r="6" spans="1:7" ht="225" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A6" s="13">
         <v>1</v>
       </c>
@@ -1933,7 +1961,7 @@
       <c r="F6" s="5"/>
       <c r="G6" s="4"/>
     </row>
-    <row r="7" spans="1:7" ht="225" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A7" s="13">
         <v>2</v>
       </c>
@@ -1950,7 +1978,7 @@
       <c r="F7" s="5"/>
       <c r="G7" s="4"/>
     </row>
-    <row r="8" spans="1:7" ht="285" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="87" x14ac:dyDescent="0.35">
       <c r="A8" s="13">
         <v>3</v>
       </c>
@@ -1967,7 +1995,7 @@
       <c r="F8" s="5"/>
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:7" ht="285" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A9" s="13">
         <v>4</v>
       </c>
@@ -1984,7 +2012,7 @@
       <c r="F9" s="5"/>
       <c r="G9" s="4"/>
     </row>
-    <row r="10" spans="1:7" ht="135" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" s="13">
         <v>5</v>
       </c>
@@ -2001,7 +2029,7 @@
       <c r="F10" s="5"/>
       <c r="G10" s="4"/>
     </row>
-    <row r="11" spans="1:7" ht="225" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A11" s="13">
         <v>6</v>
       </c>
@@ -2018,7 +2046,7 @@
       <c r="F11" s="5"/>
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:7" ht="225" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A12" s="13">
         <v>7</v>
       </c>
@@ -2035,7 +2063,7 @@
       <c r="F12" s="5"/>
       <c r="G12" s="4"/>
     </row>
-    <row r="13" spans="1:7" ht="285" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="87" x14ac:dyDescent="0.35">
       <c r="A13" s="13">
         <v>8</v>
       </c>
@@ -2052,7 +2080,7 @@
       <c r="F13" s="5"/>
       <c r="G13" s="4"/>
     </row>
-    <row r="14" spans="1:7" ht="285" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A14" s="13">
         <v>9</v>
       </c>
@@ -2069,7 +2097,7 @@
       <c r="F14" s="5"/>
       <c r="G14" s="4"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="15"/>
       <c r="B15" s="6"/>
       <c r="C15" s="7"/>
@@ -2078,7 +2106,7 @@
       <c r="F15" s="6"/>
       <c r="G15" s="6"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="17" t="s">
         <v>149</v>
       </c>
@@ -2089,7 +2117,7 @@
       <c r="F16" s="6"/>
       <c r="G16" s="6"/>
     </row>
-    <row r="17" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A17" s="13">
         <v>1</v>
       </c>
@@ -2106,7 +2134,7 @@
       <c r="F17" s="5"/>
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:7" ht="105" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A18" s="13">
         <v>2</v>
       </c>
@@ -2123,7 +2151,7 @@
       <c r="F18" s="5"/>
       <c r="G18" s="4"/>
     </row>
-    <row r="19" spans="1:7" ht="90" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="13">
         <v>3</v>
       </c>
@@ -2140,7 +2168,7 @@
       <c r="F19" s="5"/>
       <c r="G19" s="4"/>
     </row>
-    <row r="20" spans="1:7" ht="90" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="13">
         <v>4</v>
       </c>
@@ -2157,7 +2185,7 @@
       <c r="F20" s="5"/>
       <c r="G20" s="4"/>
     </row>
-    <row r="21" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="13">
         <v>5</v>
       </c>
@@ -2174,7 +2202,7 @@
       <c r="F21" s="10"/>
       <c r="G21" s="4"/>
     </row>
-    <row r="22" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A22" s="13">
         <v>6</v>
       </c>
@@ -2191,7 +2219,7 @@
       <c r="F22" s="5"/>
       <c r="G22" s="4"/>
     </row>
-    <row r="23" spans="1:7" ht="90" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A23" s="13">
         <v>6</v>
       </c>
@@ -2208,7 +2236,7 @@
       <c r="F23" s="5"/>
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A24" s="13">
         <v>7</v>
       </c>
@@ -2225,7 +2253,7 @@
       <c r="F24" s="10"/>
       <c r="G24" s="4"/>
     </row>
-    <row r="25" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A25" s="13">
         <v>8</v>
       </c>
@@ -2242,7 +2270,7 @@
       <c r="F25" s="10"/>
       <c r="G25" s="4"/>
     </row>
-    <row r="26" spans="1:7" ht="120" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A26" s="13">
         <v>9</v>
       </c>
@@ -2259,7 +2287,7 @@
       <c r="F26" s="5"/>
       <c r="G26" s="4"/>
     </row>
-    <row r="27" spans="1:7" ht="270" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" ht="87" x14ac:dyDescent="0.35">
       <c r="A27" s="13">
         <v>10</v>
       </c>
@@ -2276,7 +2304,7 @@
       <c r="F27" s="10"/>
       <c r="G27" s="4"/>
     </row>
-    <row r="28" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A28" s="13">
         <v>11</v>
       </c>
@@ -2293,7 +2321,7 @@
       <c r="F28" s="10"/>
       <c r="G28" s="4"/>
     </row>
-    <row r="29" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A29" s="13">
         <v>12</v>
       </c>
@@ -2310,7 +2338,7 @@
       <c r="F29" s="10"/>
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="1:7" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A30" s="13">
         <v>13</v>
       </c>
@@ -2339,18 +2367,17 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE440EAA-007A-486E-B4E3-7FE7599AA545}">
-  <dimension ref="A1:G33"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F36"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="55.5703125" customWidth="1"/>
-    <col min="3" max="3" width="42.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="39.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="48.7109375" customWidth="1"/>
-    <col min="6" max="6" width="50.42578125" customWidth="1"/>
-    <col min="7" max="7" width="46.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="60.08984375" customWidth="1"/>
+    <col min="3" max="3" width="42.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="44.08984375" customWidth="1"/>
+    <col min="5" max="5" width="50.453125" customWidth="1"/>
+    <col min="6" max="6" width="46.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="77.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="77.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="20" t="s">
         <v>156</v>
       </c>
@@ -2359,9 +2386,8 @@
       <c r="D1" s="20"/>
       <c r="E1" s="20"/>
       <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-    </row>
-    <row r="3" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="11" t="s">
         <v>165</v>
       </c>
@@ -2372,39 +2398,34 @@
         <v>0</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="G3" s="11" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="6"/>
       <c r="B4" s="6"/>
       <c r="C4" s="7"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="6"/>
       <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
         <v>148</v>
       </c>
       <c r="B5" s="9"/>
       <c r="C5" s="7"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="6"/>
       <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-    </row>
-    <row r="6" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="13">
         <v>1</v>
       </c>
@@ -2414,14 +2435,13 @@
       <c r="C6" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="D6" s="4"/>
-      <c r="E6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F6" s="5"/>
-      <c r="G6" s="4"/>
-    </row>
-    <row r="7" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="D6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E6" s="5"/>
+      <c r="F6" s="4"/>
+    </row>
+    <row r="7" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A7" s="13">
         <v>2</v>
       </c>
@@ -2431,14 +2451,13 @@
       <c r="C7" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="D7" s="4"/>
-      <c r="E7" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F7" s="5"/>
-      <c r="G7" s="4"/>
-    </row>
-    <row r="8" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="D7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7" s="5"/>
+      <c r="F7" s="4"/>
+    </row>
+    <row r="8" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A8" s="13">
         <v>3</v>
       </c>
@@ -2448,14 +2467,13 @@
       <c r="C8" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="D8" s="4"/>
-      <c r="E8" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F8" s="5"/>
-      <c r="G8" s="4"/>
-    </row>
-    <row r="9" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="D8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E8" s="5"/>
+      <c r="F8" s="4"/>
+    </row>
+    <row r="9" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A9" s="13">
         <v>4</v>
       </c>
@@ -2465,14 +2483,13 @@
       <c r="C9" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="D9" s="4"/>
-      <c r="E9" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F9" s="5"/>
-      <c r="G9" s="4"/>
-    </row>
-    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="D9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E9" s="5"/>
+      <c r="F9" s="4"/>
+    </row>
+    <row r="10" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="13">
         <v>5</v>
       </c>
@@ -2482,14 +2499,13 @@
       <c r="C10" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="D10" s="4"/>
-      <c r="E10" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F10" s="5"/>
-      <c r="G10" s="4"/>
-    </row>
-    <row r="11" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="D10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E10" s="5"/>
+      <c r="F10" s="4"/>
+    </row>
+    <row r="11" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11" s="13">
         <v>6</v>
       </c>
@@ -2499,14 +2515,13 @@
       <c r="C11" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="D11" s="4"/>
-      <c r="E11" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F11" s="5"/>
-      <c r="G11" s="4"/>
-    </row>
-    <row r="12" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="D11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E11" s="5"/>
+      <c r="F11" s="4"/>
+    </row>
+    <row r="12" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A12" s="13">
         <v>7</v>
       </c>
@@ -2516,14 +2531,13 @@
       <c r="C12" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="D12" s="4"/>
-      <c r="E12" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F12" s="5"/>
-      <c r="G12" s="4"/>
-    </row>
-    <row r="13" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="D12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E12" s="5"/>
+      <c r="F12" s="4"/>
+    </row>
+    <row r="13" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A13" s="13">
         <v>8</v>
       </c>
@@ -2533,14 +2547,13 @@
       <c r="C13" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="D13" s="4"/>
-      <c r="E13" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F13" s="5"/>
-      <c r="G13" s="4"/>
-    </row>
-    <row r="14" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="D13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E13" s="5"/>
+      <c r="F13" s="4"/>
+    </row>
+    <row r="14" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A14" s="13">
         <v>9</v>
       </c>
@@ -2550,316 +2563,344 @@
       <c r="C14" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="D14" s="4"/>
-      <c r="E14" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F14" s="5"/>
-      <c r="G14" s="4"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="15"/>
-      <c r="B15" s="6"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="17" t="s">
+      <c r="D14" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E14" s="5"/>
+      <c r="F14" s="4"/>
+    </row>
+    <row r="15" spans="1:6" ht="58" x14ac:dyDescent="0.35">
+      <c r="A15" s="13">
+        <v>10</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E15" s="5"/>
+      <c r="F15" s="4"/>
+    </row>
+    <row r="16" spans="1:6" ht="51.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="13">
+        <v>11</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E16" s="5"/>
+      <c r="F16" s="4"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A17" s="15"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A18" s="17" t="s">
         <v>149</v>
       </c>
-      <c r="B16" s="9"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-    </row>
-    <row r="17" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A17" s="13">
+      <c r="B18" s="9"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+    </row>
+    <row r="19" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A19" s="13">
         <v>1</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B19" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C19" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="D17" s="4"/>
-      <c r="E17" s="1" t="s">
+      <c r="D19" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="F17" s="5"/>
-      <c r="G17" s="4"/>
-    </row>
-    <row r="18" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="13">
+      <c r="E19" s="5"/>
+      <c r="F19" s="4"/>
+    </row>
+    <row r="20" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A20" s="13">
         <v>2</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B20" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C20" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="D18" s="4"/>
-      <c r="E18" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F18" s="5"/>
-      <c r="G18" s="4"/>
-    </row>
-    <row r="19" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A19" s="13">
-        <v>3</v>
-      </c>
-      <c r="B19" s="4" t="s">
+      <c r="D20" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E20" s="5"/>
+      <c r="F20" s="4"/>
+    </row>
+    <row r="21" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A21" s="13">
+        <v>3</v>
+      </c>
+      <c r="B21" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C21" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="D19" s="4"/>
-      <c r="E19" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F19" s="5"/>
-      <c r="G19" s="4"/>
-    </row>
-    <row r="20" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="13">
+      <c r="D21" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E21" s="5"/>
+      <c r="F21" s="4"/>
+    </row>
+    <row r="22" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A22" s="13">
         <v>4</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B22" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C22" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="D20" s="4"/>
-      <c r="E20" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F20" s="5"/>
-      <c r="G20" s="4"/>
-    </row>
-    <row r="21" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A21" s="13">
+      <c r="D22" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E22" s="5"/>
+      <c r="F22" s="4"/>
+    </row>
+    <row r="23" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A23" s="13">
         <v>5</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B23" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C23" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="D21" s="4"/>
-      <c r="E21" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F21" s="10"/>
-      <c r="G21" s="4"/>
-    </row>
-    <row r="22" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A22" s="13">
+      <c r="D23" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E23" s="10"/>
+      <c r="F23" s="4"/>
+    </row>
+    <row r="24" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A24" s="13">
         <v>6</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B24" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C24" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="D22" s="4"/>
-      <c r="E22" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F22" s="5"/>
-      <c r="G22" s="4"/>
-    </row>
-    <row r="23" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A23" s="13">
+      <c r="D24" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E24" s="5"/>
+      <c r="F24" s="4"/>
+    </row>
+    <row r="25" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A25" s="13">
         <v>6</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B25" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C25" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="D23" s="4"/>
-      <c r="E23" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F23" s="5"/>
-      <c r="G23" s="4"/>
-    </row>
-    <row r="24" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A24" s="13">
+      <c r="D25" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E25" s="5"/>
+      <c r="F25" s="4"/>
+    </row>
+    <row r="26" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A26" s="13">
         <v>7</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B26" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="C26" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="D24" s="4"/>
-      <c r="E24" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F24" s="10"/>
-      <c r="G24" s="4"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="13">
+      <c r="D26" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E26" s="10"/>
+      <c r="F26" s="4"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" s="13">
         <v>8</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B27" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="C27" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="D25" s="4"/>
-      <c r="E25" s="1" t="s">
+      <c r="D27" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="F25" s="10"/>
-      <c r="G25" s="4"/>
-    </row>
-    <row r="26" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A26" s="13">
+      <c r="E27" s="10"/>
+      <c r="F27" s="4"/>
+    </row>
+    <row r="28" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A28" s="13">
         <v>9</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B28" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C28" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="D26" s="4"/>
-      <c r="E26" s="1" t="s">
+      <c r="D28" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="F26" s="5"/>
-      <c r="G26" s="4"/>
-    </row>
-    <row r="27" spans="1:7" ht="60" x14ac:dyDescent="0.25">
-      <c r="A27" s="13">
+      <c r="E28" s="5"/>
+      <c r="F28" s="4"/>
+    </row>
+    <row r="29" spans="1:6" ht="58" x14ac:dyDescent="0.35">
+      <c r="A29" s="13">
         <v>10</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B29" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C29" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="D27" s="4"/>
-      <c r="E27" s="1" t="s">
+      <c r="D29" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="F27" s="10"/>
-      <c r="G27" s="4"/>
-    </row>
-    <row r="28" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A28" s="13">
+      <c r="E29" s="10"/>
+      <c r="F29" s="4"/>
+    </row>
+    <row r="30" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A30" s="13">
         <v>11</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="B30" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="C30" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="D28" s="4"/>
-      <c r="E28" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F28" s="10"/>
-      <c r="G28" s="4"/>
-    </row>
-    <row r="29" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A29" s="13">
+      <c r="D30" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E30" s="10"/>
+      <c r="F30" s="4"/>
+    </row>
+    <row r="31" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A31" s="13">
         <v>12</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="B31" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="C29" s="1" t="s">
+      <c r="C31" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="D29" s="4"/>
-      <c r="E29" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F29" s="10"/>
-      <c r="G29" s="4"/>
-    </row>
-    <row r="30" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A30" s="13">
+      <c r="D31" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E31" s="10"/>
+      <c r="F31" s="4"/>
+    </row>
+    <row r="32" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A32" s="13">
         <v>13</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="B32" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="C30" s="1" t="s">
+      <c r="C32" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="D30" s="4"/>
-      <c r="E30" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F30" s="10"/>
-      <c r="G30" s="4"/>
-    </row>
-    <row r="31" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A31" s="13">
+      <c r="D32" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E32" s="10"/>
+      <c r="F32" s="4"/>
+    </row>
+    <row r="33" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A33" s="13">
         <v>14</v>
       </c>
-      <c r="B31" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="D31" s="4"/>
-      <c r="E31" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F31" s="19"/>
-      <c r="G31" s="4"/>
-    </row>
-    <row r="32" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A32" s="13">
+      <c r="B33" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E33" s="10"/>
+      <c r="F33" s="4"/>
+    </row>
+    <row r="34" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A34" s="13">
         <v>15</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="B34" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="C34" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="D32" s="4"/>
-      <c r="E32" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F32" s="19"/>
-      <c r="G32" s="4"/>
-    </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B33" s="6"/>
-      <c r="C33" s="7"/>
-      <c r="D33" s="6"/>
-      <c r="E33" s="7"/>
-      <c r="F33" s="6"/>
-      <c r="G33" s="6"/>
+      <c r="D34" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E34" s="10"/>
+      <c r="F34" s="4"/>
+    </row>
+    <row r="35" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A35" s="13">
+        <v>16</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E35" s="10"/>
+      <c r="F35" s="4"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="B36" s="6"/>
+      <c r="C36" s="7"/>
+      <c r="D36" s="7"/>
+      <c r="E36" s="6"/>
+      <c r="F36" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -2900,15 +2941,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010039A62E282DDA434E979CD3E03185182E" ma:contentTypeVersion="33" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a6c69cf93bfe1fca5d0e373365e7fdfc">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="cea7764e-6bf9-427d-be15-e74097e0a61c" xmlns:ns3="fb9ea31f-0ab8-44ff-80d1-5777f6d9d945" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="62cb4c6faf5eab163d0c8ea23c8ff408" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -3250,6 +3282,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E53D8182-34C2-4EE5-8FD0-D750C3EB0900}">
   <ds:schemaRefs>
@@ -3270,14 +3311,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3F377113-5718-41B1-A1CE-B96F830D3573}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23B9621B-458A-4676-8042-F53348150B3A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3298,6 +3331,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3F377113-5718-41B1-A1CE-B96F830D3573}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{87867195-f2b8-4ac2-b0b6-6bb73cb33afc}" enabled="1" method="Privileged" siteId="{72f988bf-86f1-41af-91ab-2d7cd011db47}" contentBits="0" removed="0"/>

</xml_diff>